<commit_message>
epd vs e-pd benchmarks: inference_perf 6/7/8-10 runs, sglang 4img/8conc jobs, plots
Signed-off-by: Maya Barnea <mayab@il.ibm.com>
</commit_message>
<xml_diff>
--- a/benchmark/sglang/jobs_final/summary_epd_vs_e-pd.xlsx
+++ b/benchmark/sglang/jobs_final/summary_epd_vs_e-pd.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mayab/Work/AI/Routing/LLM-D/epd-benchmarks/benchmark/sglang/jobs_final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B101F31B-422A-FD45-A94B-06880556E5BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D9DA877-37B2-4443-AF79-A60D56F9C7F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-37840" yWindow="500" windowWidth="34560" windowHeight="20000" activeTab="4" xr2:uid="{527B7AD5-6E46-DC42-8E7D-6AD2838B4FAC}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="0.5-2" sheetId="8" r:id="rId4"/>
     <sheet name="Summary" sheetId="9" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -5809,10 +5809,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Summary!$I$1:$K$1</c:f>
+              <c:f>Summary!$I$1:$M$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0.5</c:v>
                 </c:pt>
@@ -5821,16 +5821,22 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Summary!$C$5:$F$5</c:f>
+              <c:f>Summary!$C$5:$G$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>2927.63</c:v>
                 </c:pt>
@@ -5842,6 +5848,9 @@
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>88693.87</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>176937.48</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5870,10 +5879,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Summary!$I$1:$K$1</c:f>
+              <c:f>Summary!$I$1:$M$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0.5</c:v>
                 </c:pt>
@@ -5882,16 +5891,22 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Summary!$I$5:$L$5</c:f>
+              <c:f>Summary!$I$5:$M$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>3058.88</c:v>
                 </c:pt>
@@ -5903,6 +5918,9 @@
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>84836.92</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>174531.19</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6667,10 +6685,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Summary!$I$1:$K$1</c:f>
+              <c:f>Summary!$I$1:$M$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0.5</c:v>
                 </c:pt>
@@ -6679,16 +6697,22 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Summary!$C$11:$F$11</c:f>
+              <c:f>Summary!$C$11:$G$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>1247.0999999999999</c:v>
                 </c:pt>
@@ -6700,6 +6724,9 @@
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>40076.39</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>123751.3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6728,10 +6755,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Summary!$I$1:$K$1</c:f>
+              <c:f>Summary!$I$1:$M$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0.5</c:v>
                 </c:pt>
@@ -6740,16 +6767,22 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Summary!$I$11:$L$11</c:f>
+              <c:f>Summary!$I$11:$M$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>1582.35</c:v>
                 </c:pt>
@@ -6761,6 +6794,9 @@
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>37488.26</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>122295.03</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7068,10 +7104,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Summary!$I$1:$K$1</c:f>
+              <c:f>Summary!$I$1:$M$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0.5</c:v>
                 </c:pt>
@@ -7080,16 +7116,22 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Summary!$C$17:$F$17</c:f>
+              <c:f>Summary!$C$17:$G$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>11.67</c:v>
                 </c:pt>
@@ -7101,6 +7143,9 @@
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>414.99</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>418.34</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7129,10 +7174,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Summary!$I$1:$K$1</c:f>
+              <c:f>Summary!$I$1:$M$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0.5</c:v>
                 </c:pt>
@@ -7141,16 +7186,22 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Summary!$I$17:$L$17</c:f>
+              <c:f>Summary!$I$17:$M$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>12.34</c:v>
                 </c:pt>
@@ -7162,6 +7213,9 @@
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>379.92</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>410.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>

</xml_diff>